<commit_message>
Restore primary SBS6 scores for MSI analyses and remove replacement readout
</commit_message>
<xml_diff>
--- a/data/Supplementary_Data_S1.xlsx
+++ b/data/Supplementary_Data_S1.xlsx
@@ -534,7 +534,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4" ht="30" customHeight="1">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -801,7 +800,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3" ht="38" customHeight="1">
       <c r="A3" s="10" t="inlineStr">
         <is>
@@ -1670,8 +1668,6 @@
         <v>0</v>
       </c>
     </row>
-    <row r="27"/>
-    <row r="28"/>
     <row r="29">
       <c r="A29" s="4" t="inlineStr">
         <is>
@@ -1681,8 +1677,6 @@
     </row>
     <row r="30"/>
     <row r="31"/>
-    <row r="32"/>
-    <row r="33"/>
     <row r="34" ht="30" customHeight="1">
       <c r="A34" s="9" t="inlineStr">
         <is>
@@ -1690,7 +1684,6 @@
         </is>
       </c>
     </row>
-    <row r="35"/>
     <row r="36" ht="38" customHeight="1">
       <c r="A36" s="10" t="inlineStr">
         <is>
@@ -2559,8 +2552,6 @@
         <v>0</v>
       </c>
     </row>
-    <row r="60"/>
-    <row r="61"/>
     <row r="62">
       <c r="A62" s="4" t="inlineStr">
         <is>
@@ -2610,7 +2601,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3" ht="38" customHeight="1">
       <c r="A3" s="10" t="inlineStr">
         <is>
@@ -3167,8 +3157,6 @@
         <v>322</v>
       </c>
     </row>
-    <row r="18"/>
-    <row r="19"/>
     <row r="20" ht="30" customHeight="1">
       <c r="A20" s="9" t="inlineStr">
         <is>
@@ -3176,7 +3164,6 @@
         </is>
       </c>
     </row>
-    <row r="21"/>
     <row r="22" ht="50" customHeight="1">
       <c r="A22" s="13" t="inlineStr">
         <is>
@@ -3281,7 +3268,7 @@
       </c>
       <c r="B30" s="4" t="inlineStr">
         <is>
-          <t>Primary-tumour sample code 01 was present in the analysed TCGA filenames. DX suffixes identify diagnostic FFPE slides, while TS/BS/MS suffixes identify frozen tissue sections [39].</t>
+          <t>Primary-tumour sample code 01 was present in the analysed TCGA filenames. DX suffixes identify diagnostic FFPE slides, while TS/BS/MS suffixes identify frozen tissue sections [38].</t>
         </is>
       </c>
     </row>
@@ -3333,8 +3320,6 @@
         </is>
       </c>
     </row>
-    <row r="35"/>
-    <row r="36"/>
     <row r="37" ht="30" customHeight="1">
       <c r="A37" s="9" t="inlineStr">
         <is>
@@ -3342,7 +3327,6 @@
         </is>
       </c>
     </row>
-    <row r="38"/>
     <row r="39" ht="65" customHeight="1">
       <c r="A39" s="13" t="inlineStr">
         <is>
@@ -3374,7 +3358,7 @@
       </c>
       <c r="G40" s="4" t="inlineStr">
         <is>
-          <t>[38] doi:10.1016/j.cell.2018.02.052
+          <t>[37] doi:10.1016/j.cell.2018.02.052
 https://gdc.cancer.gov/about-data/publications/pancanatlas</t>
         </is>
       </c>
@@ -3392,7 +3376,7 @@
       </c>
       <c r="G41" s="4" t="inlineStr">
         <is>
-          <t>[39] doi:10.1002/path.5028
+          <t>[38] doi:10.1002/path.5028
 https://docs.gdc.cancer.gov/Encyclopedia/pages/TCGA_Barcode/</t>
         </is>
       </c>

</xml_diff>